<commit_message>
Paella EN: ronda de la revisión final regenerada (4 entregables), gates G1-G9 VERDE, F2-NOTAS §9 y sha256 de §8
Sin cifras del caso, precios, costes ni ejemplos distintos; solo eventos_a2/_a3 redondeados (149 / 157). Regresión de los
7 planes en verde; sha256 Mac = VPS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LzWqvTU1jPmLwXsDXHDGWJ
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/paella-catering-business-plan/paella-catering-financial-projections.xlsx
+++ b/astro-site/public/dl/paella-catering-business-plan/paella-catering-financial-projections.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>Four 3-ring paella burners with legs (an XL 3-ring burner with tripod and regulator for pans up to 36 in (90 cm) runs about 549: Kit estimate from store prices), a rolling stand (about 399 for a 2-ring one) and wind guards. Get quotes before you buy.</t>
+          <t>Four 3-ring paella burners with legs (the XL 3-ring burner with tripod and regulator for pans up to 36 in (90 cm) runs about 549; burners for the 26-32 in pans cost less: Kit estimate from store prices), a rolling stand (about 399 for a 2-ring one) and wind guards. Get quotes before you buy.</t>
         </is>
       </c>
       <c r="E7" s="31" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="J7" s="28" t="inlineStr">
         <is>
-          <t>Servers and buffet attendants hired per event and paid hourly as W-2 employees, about one team member per 25 guests (miamigrillcatering.com). Their FTE is a fraction because they only work event hours. Treating them as 1099 contractors is a misclassification risk (FLSA; California AB5). Paid at or above the pay floor in proportion to FTE. The voluntary gratuity is theirs.</t>
+          <t>Servers and buffet attendants hired per event and paid hourly as W-2 employees, about one team member per 25 guests (miamigrillcatering.com). Their FTE is a fraction because they only work event hours. Treating them as 1099 contractors is a misclassification risk (FLSA; California AB5). Paid at or above the pay floor in proportion to FTE. The voluntary gratuity is theirs. One of them acts as event captain on the day.</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="J19" s="35" t="inlineStr">
         <is>
-          <t>Average number of people working each event: 1 on a drop-off, 2 at a backyard paella party, 3 at a company event, 4.5 at a wedding and 4 at a premium seafood event (Kit estimate). Weighted by the example mix in the Word plan, that averages about 2.5. Raise it for bigger events: the staffing sizes itself.</t>
+          <t>Average number of people working each event: 1 on a drop-off, 2 at a backyard paella party, 3 at a company event, 4.5 at a wedding and 4 at a premium seafood event (Kit estimate, about one team member per 25 guests). A full-service wedding with a tapas hour, like the calculator's example (2 paella chefs, a helper and 5 servers), takes 8: across 18 weddings that adds about 570 hours, and coverage stays above 100%. Weighted by the example mix in the Word plan, the average is about 2.5. Raise it if you staff like the calculator: the staffing sizes itself.</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3-3.5 oz (80-100 g) uncooked</t>
+          <t>3-3.5 oz (85-100 g) uncooked</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">

</xml_diff>